<commit_message>
Add Stribog clean/wind/idle/attack sets, fix tower animation bugs, add map source assets
- Stribog: clean (no-wind) rotations, separated animated wind layer, idle, bow-attack (8 dirs)
- Fix reported animation issues: Veles idle W flicker, Dazbog SW idle shield + unified spear attack, Stribog bow aim S/N/NE, Morana scythe W/NW/NE/S direction, Jarilo W/NW sickle direction
- Add PixelLab map source assets (terrain, tilesets, Rtanj, props) under Assets/Art/Map/_src
- Add animation-issues-report.md and ChatGPT map reference image

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/imena.xlsx
+++ b/imena.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mitološka mesta" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Mitološka mesta" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Mitološka mesta'!$A$1:$C$46</definedName>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,6 +36,9 @@
     <font>
       <name val="Arial"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -82,7 +85,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -93,6 +96,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -458,12 +462,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C46"/>
+  <dimension ref="A1:F46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="70" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -482,6 +489,21 @@
           <t>Kategorija</t>
         </is>
       </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Staroslovenski naziv</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Engleski naziv (tržišni)</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Izgovor (za engleske igrače)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -499,6 +521,21 @@
           <t>Onostrano / kosmološko</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Ирꙑй / Вꙑрай (Irij / Vyraj)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Vyraj — The Sunlit Shore</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>VEE-rye / EE-ree</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -516,6 +553,21 @@
           <t>Onostrano / kosmološko</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Навь (Navĭ)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Nav — The Deadlands</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>NAHV</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -533,6 +585,21 @@
           <t>Onostrano / kosmološko</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Боꙗнъ (Bojanŭ)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Buyan — The Sun Isle</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>BOO-yahn</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -550,6 +617,21 @@
           <t>Artefakt / središte sveta</t>
         </is>
       </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Алатꙑрь (Alatyrĭ)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Alatyr — The Worldstone</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>AH-lah-teer</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -567,6 +649,21 @@
           <t>Nebesko</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Сварга (Svarga)</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Svarga — The Sky Forge</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>SVAR-gah</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -584,6 +681,21 @@
           <t>Nebesko</t>
         </is>
       </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Кꙋмова слама (Kumova slama)</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>The Godfather's Way (Milky Way)</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>KOO-moh-vah SLAH-mah</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -601,6 +713,21 @@
           <t>Srpski folklor</t>
         </is>
       </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Тьмьнъ виlаѥтъ (Tĭmĭnŭ vilajetŭ)</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>The Dark Realm</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>TAHM-nee VEE-lah-yet</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -618,6 +745,21 @@
           <t>Srpska planina / epika</t>
         </is>
       </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Мирочь (Miročĭ)</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Miroch — The Vila Peak</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>MEE-rotch</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -635,6 +777,21 @@
           <t>Srpska planina / epika</t>
         </is>
       </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Ѹрвина гора (Urvina gora)</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Mount Urvina</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>OOR-vee-nah plah-NEE-nah</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -652,6 +809,21 @@
           <t>Srpska planina</t>
         </is>
       </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Проклѧтиѥ горꙑ (Proklętije gory)</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>The Accursed Mountains</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>proh-KLEH-tee-yeh</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -669,6 +841,21 @@
           <t>Srpski folklor / lokacija</t>
         </is>
       </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Дьꙗволꙗ вьсь (Dĭjavolja vĭsĭ)</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Devil's Town</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>JAH-voh-lyah VAH-rosh</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -686,6 +873,21 @@
           <t>Božanstvo-kao-mesto</t>
         </is>
       </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Триглавъ (Triglavŭ)</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Triglav — The Three-Headed Peak</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>TREE-glahv</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -703,6 +905,21 @@
           <t>Mitska daleka zemlja</t>
         </is>
       </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Тридесѧто цѣсарьство (Tridesęto cěsarĭstvo)</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>The Thirtieth Kingdom</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>TREE-deh-seh-toh TSAR-stvoh</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -720,6 +937,21 @@
           <t>Granica svetova</t>
         </is>
       </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Лѹкоморьѥ (Lukomorĭje)</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Lukomorye — The Curved Shore</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>loo-koh-MOR-yeh</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -737,6 +969,21 @@
           <t>Mitska / utopijska</t>
         </is>
       </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Бѣловодьѥ (Bělovodĭje)</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Belovodye — The White Waters</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>beh-loh-VOD-yeh</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -754,6 +1001,21 @@
           <t>Mitska daleka zemlja</t>
         </is>
       </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Китежь (Kitežĭ)</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Kitezh — The Sunken City</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>KEE-tezh</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -771,6 +1033,21 @@
           <t>Granica svetova</t>
         </is>
       </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Калиновъ мостъ (Kalinovŭ mostŭ)</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>The Kalinov Bridge</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>KAH-lee-nov MOST</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -788,6 +1065,21 @@
           <t>Granica svetova</t>
         </is>
       </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Смородина рѣка (Smorodina rěka)</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>The Smorodina — River of Fire</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>smoh-roh-DEE-nah</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -805,6 +1097,21 @@
           <t>Srpska planina</t>
         </is>
       </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Рьтьнь (Rĭtĭnĭ)</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Rtanj — The Pyramid Mountain</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>er-TAHN-y</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -822,6 +1129,21 @@
           <t>Srpska planina</t>
         </is>
       </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Бабинъ зѫбъ (Babinŭ zǫbŭ)</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>The Witch's Tooth</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>BAH-been ZOOB</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -839,6 +1161,21 @@
           <t>Planina s legendom</t>
         </is>
       </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Клекъ (Klekŭ)</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Klek — The Coven Peak</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>KLEK</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -856,6 +1193,21 @@
           <t>Srpska planina</t>
         </is>
       </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Авала (Avala)</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Avala — The Haunted Hill</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>AH-vah-lah</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -873,6 +1225,21 @@
           <t>Srpska planina</t>
         </is>
       </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Космаи (Kosmaj)</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Kosmaj — The Mystic Mount</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>KOS-my</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
@@ -890,6 +1257,21 @@
           <t>Sveto mesto u prirodi</t>
         </is>
       </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Вилино коло (Vilino kolo)</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>The Fairy Ring</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>VEE-lee-noh KOH-loh</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -907,6 +1289,21 @@
           <t>Sveto mesto u prirodi</t>
         </is>
       </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Вилино гѹмьно (Vilino gumĭno)</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>The Fairy Threshing-Floor</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>VEE-lee-noh GOOV-noh</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -924,6 +1321,21 @@
           <t>Sveto mesto u prirodi</t>
         </is>
       </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Записъ (Zapisŭ)</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>The Sacred Tree</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>ZAH-pees</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -941,6 +1353,21 @@
           <t>Sveto mesto u prirodi</t>
         </is>
       </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Гаи (Gaj)</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>The Sacred Grove</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>GUY</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
@@ -958,6 +1385,21 @@
           <t>Domen božanstva</t>
         </is>
       </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Чрьнобогъ / Бѣлобогъ (Črĭnobogŭ / Bělobogŭ)</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Chernobog &amp; Belobog — Dark and Light</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>CHER-noh-bog / BEH-loh-bog</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -975,6 +1417,21 @@
           <t>Domen božanstva</t>
         </is>
       </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Перѹновъ дѫбъ (Perunovŭ dǫbŭ)</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Perun's Oak</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>PEH-roo-nov DOOB / peh-ROO-noh-vah GOH-rah</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
@@ -992,6 +1449,21 @@
           <t>Domen božanstva</t>
         </is>
       </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Велесово полѥ (Velesovo polje)</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Veles's Field</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>VEH-leh-soh-voh POL-yeh</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1009,6 +1481,21 @@
           <t>Domen božanstva</t>
         </is>
       </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Мокошино (Mokošino)</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Mokosh's Hollow</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>moh-KOH-shee-noh</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
@@ -1026,6 +1513,21 @@
           <t>Voda</t>
         </is>
       </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Виръ (Virŭ)</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>The Whirlpool</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>VEER</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1043,6 +1545,21 @@
           <t>Voda / podzemlje</t>
         </is>
       </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Бездьнъ (Bezdĭnŭ)</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>The Abyss</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>BEZ-dahn</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
@@ -1060,6 +1577,21 @@
           <t>Voda / podzemlje</t>
         </is>
       </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Поноръ / Поникꙑ (Ponorŭ / Poniky)</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>The Sinkhole</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>POH-nor / poh-NEEK-vah</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1077,6 +1609,21 @@
           <t>Voda / ukleto</t>
         </is>
       </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Мрьтваꙗ (Mrĭtvaja)</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>The Dead Backwater</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>mer-TVAH-yah</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
@@ -1094,6 +1641,21 @@
           <t>Ukleto mesto</t>
         </is>
       </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Враждии долъ (Vraždii dolŭ)</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>The Devil's Dale</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>VRAHZH-yee DOH</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -1111,6 +1673,21 @@
           <t>Ukleto / granično</t>
         </is>
       </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Раскрьстьѥ (Raskrĭstĭje)</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>The Crossroads</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>RAHS-kersh-cheh</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
@@ -1128,6 +1705,21 @@
           <t>Ukleto mesto</t>
         </is>
       </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Разбои (Razboj)</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>The Slaughter-Ground</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>RAHZ-boy</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -1145,6 +1737,21 @@
           <t>Ukleto mesto</t>
         </is>
       </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Мрьтво брьдо / Гологлавъ (Mrĭtvo brĭdo / Gologlavŭ)</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Deadhill / Baldcrown</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>MER-tvoh BER-doh / GOH-loh-glahv</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
@@ -1162,6 +1769,21 @@
           <t>Mitska daleka zemlja</t>
         </is>
       </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Индиꙗ (Indija)</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Mythic India — Land of Plenty</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>EEN-dee-yah</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -1179,6 +1801,21 @@
           <t>Lokacija / zvučno ime</t>
         </is>
       </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Златоборъ (Zlatoborŭ)</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Zlatibor — The Golden Pines</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>ZLAH-tee-bor</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
@@ -1196,6 +1833,21 @@
           <t>Mitska zemlja</t>
         </is>
       </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Дѣвичьско цѣсарьство (Děvičĭsko cěsarĭstvo)</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>The Maiden Kingdom</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>DEH-veetch-yeh TSAR-stvoh</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -1213,6 +1865,21 @@
           <t>Atmosferično ime</t>
         </is>
       </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Навьѥ (Navĭje)</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Navlje — The Place of the Dead</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>NAHV-lyeh</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
@@ -1230,6 +1897,21 @@
           <t>Atmosferično ime</t>
         </is>
       </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Сѫтонъ (Sǫtonŭ)</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Duskfall</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>SOO-ton</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -1245,6 +1927,21 @@
       <c r="C46" s="2" t="inlineStr">
         <is>
           <t>Atmosferično ime</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Глота (Glota)</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Glota — The Deep Dark</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>GLOH-tah</t>
         </is>
       </c>
     </row>

</xml_diff>